<commit_message>
feat: complete advanced workbook import diagnostics
</commit_message>
<xml_diff>
--- a/test-fixtures/problematic-import.xlsx
+++ b/test-fixtures/problematic-import.xlsx
@@ -77,6 +77,28 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ResumoPorCidade">
+  <location ref="I4:L10"/>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="VendasImportadas" displayName="VendasImportadas" ref="A4:G8">
+  <tableColumns count="7">
+    <tableColumn id="1" name="Data"/>
+    <tableColumn id="2" name="Cidade"/>
+    <tableColumn id="3" name="CPF"/>
+    <tableColumn id="4" name="Categoria"/>
+    <tableColumn id="5" name="Faturamento"/>
+    <tableColumn id="6" name="Taxa"/>
+    <tableColumn id="7" name="Total calculado">
+      <calculatedColumnFormula>Faturamento</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -534,6 +556,10 @@
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
+  <tableParts count="1">
+    <tablePart r:id="rIdTable"/>
+  </tableParts>
+  <pivotTableDefinition r:id="rIdPivot"/>
 </worksheet>
 </file>
 

</xml_diff>